<commit_message>
primary energy and emission factors input data corrected
Value 0 was needed for heating or cooling fuel type 'None', 'NoHeating' and 'NoCooling'
</commit_message>
<xml_diff>
--- a/src/dibs_data/data/LCA/Primary_energy_and_emission_factors.xlsx
+++ b/src/dibs_data/data/LCA/Primary_energy_and_emission_factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\BE_data\DibsData_101_NormProfiles\NEW_AM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F6801AB-4F6A-4676-A4B6-400A2AA4D60C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE04C8F6-3786-4860-88E4-0A88C7EF3531}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13425"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Primary_energy_and_emission_fac" sheetId="1" r:id="rId1"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -988,7 +988,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1572,6 +1572,12 @@
       <c r="E31" t="s">
         <v>39</v>
       </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -1589,6 +1595,12 @@
       <c r="E32" t="s">
         <v>39</v>
       </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
@@ -1628,6 +1640,12 @@
       </c>
       <c r="E34" t="s">
         <v>39</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjusted Primary Energy Factors for biogas
primary energy factors added for biogas and biooil. PEF for electricity in 2040 adjusted.
</commit_message>
<xml_diff>
--- a/src/dibs_data/data/LCA/Primary_energy_and_emission_factors.xlsx
+++ b/src/dibs_data/data/LCA/Primary_energy_and_emission_factors.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\BE_data\DibsData_101_NormProfiles\NEW_AM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\André\Documents\GitHub\DibsData\src\dibs_data\data\LCA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE04C8F6-3786-4860-88E4-0A88C7EF3531}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C71EC776-1AC6-40E0-B5B0-929AF3B94FB7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1134,6 +1134,12 @@
       <c r="E7" t="s">
         <v>8</v>
       </c>
+      <c r="F7">
+        <v>0.8</v>
+      </c>
+      <c r="G7">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1168,6 +1174,12 @@
       <c r="E9" t="s">
         <v>8</v>
       </c>
+      <c r="F9">
+        <v>0.8</v>
+      </c>
+      <c r="G9">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1202,6 +1214,12 @@
       <c r="E11" t="s">
         <v>8</v>
       </c>
+      <c r="F11">
+        <v>0.8</v>
+      </c>
+      <c r="G11">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1237,10 +1255,10 @@
         <v>8</v>
       </c>
       <c r="F13">
-        <v>1.1000000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="G13">
-        <v>1.1000000000000001</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1536,7 +1554,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="G29">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>